<commit_message>
Nation-Daten: recompute-1950s-road-f1.js + Indy-freier F1-Blend (Deliverable + Excel regeneriert)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FyTWK1EifL9fGNn28seeRn
</commit_message>
<xml_diff>
--- a/fable-deliverables/nation-data/nation-frequency-by-decade.xlsx
+++ b/fable-deliverables/nation-data/nation-frequency-by-decade.xlsx
@@ -7793,10 +7793,10 @@
         <v>USA</v>
       </c>
       <c r="B2">
-        <v>30.22</v>
+        <v>16.42</v>
       </c>
       <c r="C2">
-        <v>19.4</v>
+        <v>18.49</v>
       </c>
       <c r="D2">
         <v>14.4</v>
@@ -7817,7 +7817,7 @@
         <v>15.78</v>
       </c>
       <c r="J2">
-        <v>16.17</v>
+        <v>14.33</v>
       </c>
     </row>
     <row r="3">
@@ -7825,10 +7825,10 @@
         <v>FRA</v>
       </c>
       <c r="B3">
-        <v>12.27</v>
+        <v>13.85</v>
       </c>
       <c r="C3">
-        <v>9.94</v>
+        <v>9.99</v>
       </c>
       <c r="D3">
         <v>11.33</v>
@@ -7849,7 +7849,7 @@
         <v>8.98</v>
       </c>
       <c r="J3">
-        <v>9.19</v>
+        <v>9.39</v>
       </c>
     </row>
     <row r="4">
@@ -7857,10 +7857,10 @@
         <v>GBR</v>
       </c>
       <c r="B4">
-        <v>18.11</v>
+        <v>23.04</v>
       </c>
       <c r="C4">
-        <v>15.55</v>
+        <v>15.81</v>
       </c>
       <c r="D4">
         <v>11.78</v>
@@ -7881,7 +7881,7 @@
         <v>12.71</v>
       </c>
       <c r="J4">
-        <v>12.67</v>
+        <v>13.32</v>
       </c>
     </row>
     <row r="5">
@@ -7889,10 +7889,10 @@
         <v>ITA</v>
       </c>
       <c r="B5">
-        <v>10.71</v>
+        <v>12.41</v>
       </c>
       <c r="C5">
-        <v>9.74</v>
+        <v>9.87</v>
       </c>
       <c r="D5">
         <v>9.86</v>
@@ -7913,7 +7913,7 @@
         <v>3.36</v>
       </c>
       <c r="J5">
-        <v>9.57</v>
+        <v>9.8</v>
       </c>
     </row>
     <row r="6">
@@ -7921,10 +7921,10 @@
         <v>GER</v>
       </c>
       <c r="B6">
-        <v>7.51</v>
+        <v>9.28</v>
       </c>
       <c r="C6">
-        <v>5.63</v>
+        <v>5.67</v>
       </c>
       <c r="D6">
         <v>3.91</v>
@@ -7945,7 +7945,7 @@
         <v>5.13</v>
       </c>
       <c r="J6">
-        <v>7.06</v>
+        <v>7.29</v>
       </c>
     </row>
     <row r="7">
@@ -7985,10 +7985,10 @@
         <v>ARG</v>
       </c>
       <c r="B8">
-        <v>3.19</v>
+        <v>4.07</v>
       </c>
       <c r="C8">
-        <v>2.69</v>
+        <v>2.72</v>
       </c>
       <c r="D8">
         <v>2.46</v>
@@ -8009,7 +8009,7 @@
         <v>2.08</v>
       </c>
       <c r="J8">
-        <v>2.72</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="9">
@@ -8017,7 +8017,7 @@
         <v>ESP</v>
       </c>
       <c r="B9">
-        <v>1.26</v>
+        <v>1.45</v>
       </c>
       <c r="C9">
         <v>1.56</v>
@@ -8041,7 +8041,7 @@
         <v>7.17</v>
       </c>
       <c r="J9">
-        <v>3.72</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="10">
@@ -8049,7 +8049,7 @@
         <v>BRA</v>
       </c>
       <c r="B10">
-        <v>0.85</v>
+        <v>1.1</v>
       </c>
       <c r="C10">
         <v>0.31</v>
@@ -8073,7 +8073,7 @@
         <v>2</v>
       </c>
       <c r="J10">
-        <v>4.05</v>
+        <v>4.08</v>
       </c>
     </row>
     <row r="11">
@@ -8081,10 +8081,10 @@
         <v>AUS</v>
       </c>
       <c r="B11">
-        <v>1.23</v>
+        <v>1.48</v>
       </c>
       <c r="C11">
-        <v>1.97</v>
+        <v>1.98</v>
       </c>
       <c r="D11">
         <v>3.32</v>
@@ -8105,7 +8105,7 @@
         <v>5.02</v>
       </c>
       <c r="J11">
-        <v>3.18</v>
+        <v>3.21</v>
       </c>
     </row>
     <row r="12">
@@ -8113,10 +8113,10 @@
         <v>SWE</v>
       </c>
       <c r="B12">
-        <v>0.73</v>
+        <v>0.79</v>
       </c>
       <c r="C12">
-        <v>1.2</v>
+        <v>1.19</v>
       </c>
       <c r="D12">
         <v>3.71</v>
@@ -8145,10 +8145,10 @@
         <v>SUI</v>
       </c>
       <c r="B13">
-        <v>2.11</v>
+        <v>2.61</v>
       </c>
       <c r="C13">
-        <v>4.13</v>
+        <v>4.19</v>
       </c>
       <c r="D13">
         <v>2.79</v>
@@ -8169,7 +8169,7 @@
         <v>0.38</v>
       </c>
       <c r="J13">
-        <v>1.9</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="14">
@@ -8177,10 +8177,10 @@
         <v>BEL</v>
       </c>
       <c r="B14">
-        <v>2.79</v>
+        <v>3.61</v>
       </c>
       <c r="C14">
-        <v>1.7</v>
+        <v>1.71</v>
       </c>
       <c r="D14">
         <v>2.5</v>
@@ -8201,7 +8201,7 @@
         <v>0.56</v>
       </c>
       <c r="J14">
-        <v>1.64</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="15">
@@ -8212,7 +8212,7 @@
         <v>0.39</v>
       </c>
       <c r="C15">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="D15">
         <v>1.9</v>
@@ -8244,7 +8244,7 @@
         <v>0.93</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="D16">
         <v>1.53</v>
@@ -8265,7 +8265,7 @@
         <v>0.38</v>
       </c>
       <c r="J16">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="17">
@@ -8276,7 +8276,7 @@
         <v>0.47</v>
       </c>
       <c r="C17">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="D17">
         <v>1.28</v>
@@ -8305,7 +8305,7 @@
         <v>NED</v>
       </c>
       <c r="B18">
-        <v>0.76</v>
+        <v>0.95</v>
       </c>
       <c r="C18">
         <v>0.94</v>
@@ -8329,7 +8329,7 @@
         <v>4.36</v>
       </c>
       <c r="J18">
-        <v>2.14</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="19">
@@ -8340,7 +8340,7 @@
         <v>0.43</v>
       </c>
       <c r="C19">
-        <v>3.34</v>
+        <v>3.39</v>
       </c>
       <c r="D19">
         <v>2.08</v>
@@ -8361,7 +8361,7 @@
         <v>4.81</v>
       </c>
       <c r="J19">
-        <v>2.45</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="20">
@@ -8372,7 +8372,7 @@
         <v>0.53</v>
       </c>
       <c r="C20">
-        <v>1.92</v>
+        <v>1.93</v>
       </c>
       <c r="D20">
         <v>3.16</v>
@@ -8404,7 +8404,7 @@
         <v>0.42</v>
       </c>
       <c r="C21">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="D21">
         <v>0.9</v>
@@ -8433,10 +8433,10 @@
         <v>NZL</v>
       </c>
       <c r="B22">
-        <v>0.35</v>
+        <v>0.41</v>
       </c>
       <c r="C22">
-        <v>1.84</v>
+        <v>1.86</v>
       </c>
       <c r="D22">
         <v>1.56</v>
@@ -8457,7 +8457,7 @@
         <v>0.25</v>
       </c>
       <c r="J22">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="23">
@@ -8529,10 +8529,10 @@
         <v>POR</v>
       </c>
       <c r="B25">
-        <v>0.35</v>
+        <v>0.41</v>
       </c>
       <c r="C25">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="D25">
         <v>0.47</v>
@@ -8553,7 +8553,7 @@
         <v>0.25</v>
       </c>
       <c r="J25">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="26">
@@ -8564,7 +8564,7 @@
         <v>0.07</v>
       </c>
       <c r="C26">
-        <v>1.35</v>
+        <v>1.37</v>
       </c>
       <c r="D26">
         <v>0.72</v>
@@ -8585,7 +8585,7 @@
         <v>0.94</v>
       </c>
       <c r="J26">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="27">
@@ -8596,7 +8596,7 @@
         <v>0.09</v>
       </c>
       <c r="C27">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="D27">
         <v>0.88</v>
@@ -8628,7 +8628,7 @@
         <v>0.37</v>
       </c>
       <c r="C28">
-        <v>5.47</v>
+        <v>5.58</v>
       </c>
       <c r="D28">
         <v>2.23</v>
@@ -8649,7 +8649,7 @@
         <v>0.44</v>
       </c>
       <c r="J28">
-        <v>1.27</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="29">
@@ -8753,10 +8753,10 @@
         <v>IRL</v>
       </c>
       <c r="B32">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="C32">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="D32">
         <v>0.59</v>
@@ -8777,7 +8777,7 @@
         <v>0.12</v>
       </c>
       <c r="J32">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="33">
@@ -8820,7 +8820,7 @@
         <v>0.02</v>
       </c>
       <c r="C34">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D34">
         <v>0.22</v>
@@ -8884,7 +8884,7 @@
         <v>0.15</v>
       </c>
       <c r="C36">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="D36">
         <v>0.09</v>
@@ -8945,7 +8945,7 @@
         <v>THA</v>
       </c>
       <c r="B38">
-        <v>0.17</v>
+        <v>0.23</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -8969,7 +8969,7 @@
         <v>2.61</v>
       </c>
       <c r="J38">
-        <v>0.48</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="39">
@@ -8980,7 +8980,7 @@
         <v>0.02</v>
       </c>
       <c r="C39">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D39">
         <v>0.09</v>
@@ -9044,7 +9044,7 @@
         <v>0.1</v>
       </c>
       <c r="C41">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="D41">
         <v>0.39</v>
@@ -9065,7 +9065,7 @@
         <v>0</v>
       </c>
       <c r="J41">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="42">
@@ -9076,7 +9076,7 @@
         <v>0.09</v>
       </c>
       <c r="C42">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D42">
         <v>0.13</v>
@@ -9233,10 +9233,10 @@
         <v>URU</v>
       </c>
       <c r="B47">
-        <v>0.66</v>
+        <v>0.91</v>
       </c>
       <c r="C47">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D47">
         <v>0.05</v>
@@ -9257,7 +9257,7 @@
         <v>0.25</v>
       </c>
       <c r="J47">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="48">
@@ -9265,7 +9265,7 @@
         <v>MON</v>
       </c>
       <c r="B48">
-        <v>0.34</v>
+        <v>0.46</v>
       </c>
       <c r="C48">
         <v>0</v>
@@ -9289,7 +9289,7 @@
         <v>2.98</v>
       </c>
       <c r="J48">
-        <v>0.67</v>
+        <v>0.69</v>
       </c>
     </row>
     <row r="49">
@@ -9460,7 +9460,7 @@
         <v>0.09</v>
       </c>
       <c r="C54">
-        <v>1.13</v>
+        <v>1.15</v>
       </c>
       <c r="D54">
         <v>0.09</v>
@@ -9524,7 +9524,7 @@
         <v>0</v>
       </c>
       <c r="C56">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -9553,10 +9553,10 @@
         <v>MAR</v>
       </c>
       <c r="B57">
-        <v>0.17</v>
+        <v>0.23</v>
       </c>
       <c r="C57">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D57">
         <v>0</v>
@@ -9577,7 +9577,7 @@
         <v>0.19</v>
       </c>
       <c r="J57">
-        <v>0.07</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="58">
@@ -9652,7 +9652,7 @@
         <v>0.02</v>
       </c>
       <c r="C60">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D60">
         <v>0.05</v>
@@ -9780,7 +9780,7 @@
         <v>0.02</v>
       </c>
       <c r="C64">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -9940,7 +9940,7 @@
         <v>0</v>
       </c>
       <c r="C69">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D69">
         <v>0.05</v>
@@ -10004,7 +10004,7 @@
         <v>0</v>
       </c>
       <c r="C71">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D71">
         <v>0</v>
@@ -10036,7 +10036,7 @@
         <v>0</v>
       </c>
       <c r="C72">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D72">
         <v>0.05</v>
@@ -10484,7 +10484,7 @@
         <v>0</v>
       </c>
       <c r="C86">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D86">
         <v>0.05</v>
@@ -10516,7 +10516,7 @@
         <v>0</v>
       </c>
       <c r="C87">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D87">
         <v>0.05</v>
@@ -10996,7 +10996,7 @@
         <v>0</v>
       </c>
       <c r="C102">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D102">
         <v>0</v>

</xml_diff>